<commit_message>
Update Joy Gomes' role to match spreadsheet
Role/Title changed from "Thesis Chair" to "ABAAS Masters Student" in the
team database; synced to her homepage card and team.html listing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/PIRL-Team-Database.xlsx
+++ b/data/PIRL-Team-Database.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentuml-my.sharepoint.com/personal/jiabin_shen_uml_edu/Documents/Research/Lab/Website/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentuml-my.sharepoint.com/personal/jiabin_shen_uml_edu/Documents/Research/Lab/Website/github/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_9585E1FC1DC8A59F83486DA983AFA05085CCC031" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAE0FAB5-0CE7-9443-8311-9E09758A0A31}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_9585E1FC1DC8A59F83486DA983AFA05085CCC031" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B3F3060-8C85-DB48-A0ED-73D5CC6FBC04}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="38400" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -265,9 +265,6 @@
     <t>Joy Gomes</t>
   </si>
   <si>
-    <t>Thesis Chair</t>
-  </si>
-  <si>
     <t>Master's – Applied Behavior Analysis &amp; Autism Studies</t>
   </si>
   <si>
@@ -629,6 +626,9 @@
   </si>
   <si>
     <t>If a photo filename is left blank, that person will simply show initials — nothing breaks.</t>
+  </si>
+  <si>
+    <t>ABAAS Masters Student</t>
   </si>
 </sst>
 </file>
@@ -738,7 +738,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -757,6 +757,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1070,12 +1071,12 @@
   <sheetData>
     <row r="2" spans="2:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.2">
@@ -1083,7 +1084,7 @@
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
@@ -1091,52 +1092,52 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -1144,126 +1145,126 @@
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="16" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C29" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C31" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C34" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="16" x14ac:dyDescent="0.2">
       <c r="B36" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C39" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C40" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C41" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C42" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B44" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C45" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C46" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="C47" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1763,8 +1764,8 @@
       <c r="C13" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>80</v>
+      <c r="D13" s="12" t="s">
+        <v>201</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>19</v>
@@ -1778,10 +1779,10 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="O13" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>82</v>
       </c>
       <c r="P13" s="11" t="s">
         <v>43</v>
@@ -1795,10 +1796,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>34</v>
@@ -1812,10 +1813,10 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="O14" s="11" t="s">
         <v>85</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>86</v>
       </c>
       <c r="P14" s="11" t="s">
         <v>63</v>
@@ -1829,10 +1830,10 @@
         <v>12</v>
       </c>
       <c r="C15" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>88</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>34</v>
@@ -1849,7 +1850,7 @@
         <v>41</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P15" s="11" t="s">
         <v>63</v>
@@ -1863,10 +1864,10 @@
         <v>13</v>
       </c>
       <c r="C16" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>90</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>91</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>34</v>
@@ -1883,7 +1884,7 @@
         <v>41</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P16" s="11" t="s">
         <v>63</v>
@@ -1897,10 +1898,10 @@
         <v>14</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>34</v>
@@ -1917,7 +1918,7 @@
         <v>41</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P17" s="11" t="s">
         <v>63</v>
@@ -1931,10 +1932,10 @@
         <v>15</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>34</v>
@@ -1951,7 +1952,7 @@
         <v>41</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P18" s="11" t="s">
         <v>63</v>
@@ -1965,10 +1966,10 @@
         <v>16</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>34</v>
@@ -1985,7 +1986,7 @@
         <v>41</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P19" s="11" t="s">
         <v>63</v>
@@ -1999,10 +2000,10 @@
         <v>17</v>
       </c>
       <c r="C20" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>98</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>99</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>34</v>
@@ -2016,7 +2017,7 @@
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O20" s="11" t="s">
         <v>78</v>
@@ -2033,10 +2034,10 @@
         <v>18</v>
       </c>
       <c r="C21" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>101</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>34</v>
@@ -2053,7 +2054,7 @@
         <v>58</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P21" s="11" t="s">
         <v>63</v>
@@ -2067,10 +2068,10 @@
         <v>19</v>
       </c>
       <c r="C22" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>103</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>104</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>34</v>
@@ -2087,7 +2088,7 @@
         <v>58</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P22" s="11" t="s">
         <v>63</v>
@@ -2101,10 +2102,10 @@
         <v>20</v>
       </c>
       <c r="C23" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>34</v>
@@ -2121,7 +2122,7 @@
         <v>58</v>
       </c>
       <c r="O23" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P23" s="11" t="s">
         <v>63</v>
@@ -2135,10 +2136,10 @@
         <v>21</v>
       </c>
       <c r="C24" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>108</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>109</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>34</v>
@@ -2155,7 +2156,7 @@
         <v>58</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P24" s="11" t="s">
         <v>63</v>
@@ -2169,10 +2170,10 @@
         <v>22</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>34</v>
@@ -2189,7 +2190,7 @@
         <v>58</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P25" s="11" t="s">
         <v>63</v>
@@ -2203,10 +2204,10 @@
         <v>23</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>34</v>
@@ -2223,7 +2224,7 @@
         <v>58</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P26" s="11" t="s">
         <v>63</v>
@@ -2237,10 +2238,10 @@
         <v>24</v>
       </c>
       <c r="C27" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>34</v>
@@ -2257,7 +2258,7 @@
         <v>58</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P27" s="11" t="s">
         <v>63</v>
@@ -2271,10 +2272,10 @@
         <v>25</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>34</v>
@@ -2291,7 +2292,7 @@
         <v>58</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P28" s="11" t="s">
         <v>63</v>
@@ -2305,10 +2306,10 @@
         <v>26</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>34</v>
@@ -2325,7 +2326,7 @@
         <v>58</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P29" s="11" t="s">
         <v>63</v>
@@ -2339,10 +2340,10 @@
         <v>27</v>
       </c>
       <c r="C30" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>117</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>118</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>34</v>
@@ -2359,7 +2360,7 @@
         <v>58</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P30" s="11" t="s">
         <v>63</v>
@@ -2373,10 +2374,10 @@
         <v>28</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>34</v>
@@ -2393,7 +2394,7 @@
         <v>58</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P31" s="11" t="s">
         <v>63</v>
@@ -2407,10 +2408,10 @@
         <v>29</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>34</v>
@@ -2441,10 +2442,10 @@
         <v>30</v>
       </c>
       <c r="C33" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="11" t="s">
         <v>121</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>122</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>34</v>
@@ -2461,7 +2462,7 @@
         <v>58</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P33" s="11" t="s">
         <v>63</v>
@@ -2475,10 +2476,10 @@
         <v>31</v>
       </c>
       <c r="C34" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>123</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>124</v>
       </c>
       <c r="E34" s="11" t="s">
         <v>34</v>
@@ -2495,7 +2496,7 @@
         <v>58</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P34" s="11" t="s">
         <v>63</v>
@@ -2509,10 +2510,10 @@
         <v>32</v>
       </c>
       <c r="C35" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>126</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>127</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>34</v>
@@ -2529,7 +2530,7 @@
         <v>58</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P35" s="11" t="s">
         <v>63</v>
@@ -2543,10 +2544,10 @@
         <v>33</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>34</v>
@@ -2563,7 +2564,7 @@
         <v>58</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P36" s="11" t="s">
         <v>63</v>
@@ -2577,10 +2578,10 @@
         <v>34</v>
       </c>
       <c r="C37" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="D37" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>130</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>34</v>
@@ -2597,7 +2598,7 @@
         <v>58</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P37" s="11" t="s">
         <v>63</v>
@@ -2611,10 +2612,10 @@
         <v>35</v>
       </c>
       <c r="C38" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D38" s="11" t="s">
         <v>131</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>132</v>
       </c>
       <c r="E38" s="11" t="s">
         <v>34</v>
@@ -2628,10 +2629,10 @@
       <c r="L38" s="11"/>
       <c r="M38" s="11"/>
       <c r="N38" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P38" s="11" t="s">
         <v>63</v>
@@ -2645,10 +2646,10 @@
         <v>36</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>34</v>
@@ -2662,7 +2663,7 @@
       <c r="L39" s="11"/>
       <c r="M39" s="11"/>
       <c r="N39" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="O39" s="11" t="s">
         <v>51</v>
@@ -2679,10 +2680,10 @@
         <v>37</v>
       </c>
       <c r="C40" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D40" s="11" t="s">
         <v>136</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>137</v>
       </c>
       <c r="E40" s="11" t="s">
         <v>34</v>
@@ -2696,7 +2697,7 @@
       <c r="L40" s="11"/>
       <c r="M40" s="11"/>
       <c r="N40" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O40" s="11" t="s">
         <v>51</v>
@@ -2735,18 +2736,18 @@
   <sheetData>
     <row r="2" spans="2:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
@@ -2773,12 +2774,12 @@
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -2797,7 +2798,7 @@
   <sheetData>
     <row r="2" spans="2:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.2">
@@ -2805,12 +2806,12 @@
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.2">
@@ -2818,7 +2819,7 @@
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.2">
@@ -2826,12 +2827,12 @@
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.2">
@@ -2839,7 +2840,7 @@
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.2">
@@ -2847,17 +2848,17 @@
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.2">
@@ -2865,12 +2866,12 @@
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.2">
@@ -2878,7 +2879,7 @@
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.2">
@@ -2886,12 +2887,12 @@
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B24" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.2">
@@ -2899,12 +2900,12 @@
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B26" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B27" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.2">
@@ -2912,7 +2913,7 @@
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B29" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sort team.html alumni chronologically instead of by manual order
Each Degree Level group now sorts by parsed Years in Lab (end year
descending, then start year, then name) so new alumni rows slot into
the right position automatically. Current Members still sort by the
spreadsheet's manual Order column. Joy Gomes' card role text and focus
fallback are updated to match the latest spreadsheet, and ITGcard now
skips the Current Focus label gracefully when focus is blank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/PIRL-Team-Database.xlsx
+++ b/data/PIRL-Team-Database.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C52"/>
+  <dimension ref="B2:C59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -519,11 +519,14 @@
   </cols>
   <sheetData>
     <row r="2" ht="20" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Pediatric Injury Research Lab — Team Database</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="10" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
@@ -531,9 +534,11 @@
           <t>How this works</t>
         </is>
       </c>
+      <c r="C4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="3" t="n"/>
+      <c r="C5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -541,9 +546,11 @@
           <t>This workbook is the single source of truth for the 'Meet the Lab' section on your website.</t>
         </is>
       </c>
+      <c r="C6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="n"/>
+      <c r="C7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
@@ -826,6 +833,48 @@
       <c r="C52" s="10" t="inlineStr">
         <is>
           <t>(not primary mentor) are excluded. Source: Shen CV, Student Mentoring section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>6.  For Alumni, the website sorts automatically by 'Years in Lab' (most recent</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>first) within each Degree Level -- the 'Order' column is NOT used for Alumni, only</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>for Current Members. Add a new alumni row with the correct Years and it will appear</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>in the right place automatically -- no renumbering needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>An open-ended range like "2024-" means still ongoing -- if someone is still active,</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>they belong in Current Members, not Alumni.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1119,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
@@ -1139,7 +1188,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
@@ -1208,7 +1257,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
@@ -1383,7 +1432,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
@@ -1436,7 +1485,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
@@ -1489,7 +1538,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
@@ -1542,7 +1591,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
@@ -1595,7 +1644,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
@@ -1604,7 +1653,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Master's Thesis</t>
+          <t>MS in Applied Behavior Analysis &amp; Autism Studies · Master's Thesis</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -1620,26 +1669,10 @@
       <c r="K13" s="12" t="n"/>
       <c r="L13" s="12" t="n"/>
       <c r="M13" s="12" t="n"/>
-      <c r="N13" s="12" t="inlineStr">
-        <is>
-          <t>Master's</t>
-        </is>
-      </c>
-      <c r="O13" s="12" t="inlineStr">
-        <is>
-          <t>Applied Behavior Analysis &amp; Autism Studies</t>
-        </is>
-      </c>
-      <c r="P13" s="12" t="inlineStr">
-        <is>
-          <t>2024–</t>
-        </is>
-      </c>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12" t="n"/>
+      <c r="P13" s="12" t="n"/>
+      <c r="Q13" s="12" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1648,7 +1681,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
@@ -1701,7 +1734,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
@@ -1754,7 +1787,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
@@ -1807,7 +1840,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
@@ -1860,7 +1893,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
@@ -1913,7 +1946,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
@@ -1966,7 +1999,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
@@ -2015,7 +2048,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
@@ -2052,7 +2085,7 @@
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>2024–</t>
+          <t>2024–2025</t>
         </is>
       </c>
       <c r="Q21" s="12" t="inlineStr">
@@ -2068,7 +2101,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
@@ -2105,7 +2138,7 @@
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
-          <t>2025–</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="Q22" s="12" t="inlineStr">
@@ -2121,7 +2154,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
@@ -2174,7 +2207,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
@@ -2227,7 +2260,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
@@ -2280,7 +2313,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
@@ -2333,7 +2366,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
@@ -2386,7 +2419,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
@@ -2439,7 +2472,7 @@
         </is>
       </c>
       <c r="B29" s="12" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
@@ -2492,7 +2525,7 @@
         </is>
       </c>
       <c r="B30" s="12" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
@@ -2545,7 +2578,7 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
@@ -2598,7 +2631,7 @@
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
@@ -2651,7 +2684,7 @@
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
@@ -2704,7 +2737,7 @@
         </is>
       </c>
       <c r="B34" s="12" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
@@ -2757,7 +2790,7 @@
         </is>
       </c>
       <c r="B35" s="12" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
@@ -2810,7 +2843,7 @@
         </is>
       </c>
       <c r="B36" s="12" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
@@ -2863,7 +2896,7 @@
         </is>
       </c>
       <c r="B37" s="12" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
@@ -2916,7 +2949,7 @@
         </is>
       </c>
       <c r="B38" s="12" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
@@ -2969,7 +3002,7 @@
         </is>
       </c>
       <c r="B39" s="12" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
@@ -3022,7 +3055,7 @@
         </is>
       </c>
       <c r="B40" s="12" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>

</xml_diff>